<commit_message>
CBS ledger fixes, UI polish, and release v1.0.9
</commit_message>
<xml_diff>
--- a/bill format.xlsx
+++ b/bill format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\amit sagu\awagaman project\ATL ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C5BFEE-26E9-4B72-8990-F39EFE20457E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF2260A-08D8-47E3-9BC1-BB8EB9A1AB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{3AFE51C9-C4A8-42BB-8FE9-153B9C434294}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>To</t>
   </si>
@@ -42,24 +42,9 @@
     <t>Bill No.</t>
   </si>
   <si>
-    <t>FBD 25-26/ 1002</t>
-  </si>
-  <si>
-    <t>M/s  Kadence Automation and Robotic Systems (Consignor Name from bilty)</t>
-  </si>
-  <si>
-    <t>Plot No.166 , Shed No. 1 &amp; 2, Badkhal- Pali Road, Village- Bhankari, Faridabad (consignor from bilty)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Date :</t>
   </si>
   <si>
-    <t>30.03.2026</t>
-  </si>
-  <si>
-    <t>Party GST No.    06AATFK3508J1Z1              State Code : 06 (this is only starting two digit of gst no.)</t>
-  </si>
-  <si>
     <t>C/N No</t>
   </si>
   <si>
@@ -90,55 +75,13 @@
     <t>To……..</t>
   </si>
   <si>
-    <t>30.03.26</t>
-  </si>
-  <si>
-    <t>KS/25-26/1688</t>
-  </si>
-  <si>
-    <t>HR38AJ0683</t>
-  </si>
-  <si>
-    <t>Faridabad</t>
-  </si>
-  <si>
-    <t>Ghaziabad</t>
-  </si>
-  <si>
-    <t>Canter 22'</t>
-  </si>
-  <si>
-    <t>Settle</t>
-  </si>
-  <si>
-    <t>KS/25-26/1695</t>
-  </si>
-  <si>
-    <t>HR46F3857</t>
-  </si>
-  <si>
-    <t>Kharkhoda</t>
-  </si>
-  <si>
     <t xml:space="preserve">  Rupees in Words :</t>
   </si>
   <si>
-    <t>Twenty Nine Thousand Only</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>Encl…………Ack / ment</t>
   </si>
   <si>
     <t xml:space="preserve">                         For Awagaman Trans Logistics </t>
-  </si>
-  <si>
-    <t>Hamali</t>
-  </si>
-  <si>
-    <t>Detention</t>
   </si>
 </sst>
 </file>
@@ -428,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -538,101 +481,98 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -973,121 +913,111 @@
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="2:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="58" t="s">
+      <c r="C5" s="47"/>
+      <c r="D5" s="48"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="51"/>
+      <c r="L5" s="51"/>
+    </row>
+    <row r="6" spans="2:13" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="46"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="4"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B7" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="F5" s="62" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="62"/>
-      <c r="J5" s="62"/>
-      <c r="K5" s="62"/>
-      <c r="L5" s="62"/>
-    </row>
-    <row r="6" spans="2:13" ht="16.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="57"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="63" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="4"/>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B7" s="56" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="64" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="65"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="54"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="63"/>
-      <c r="G7" s="63"/>
-      <c r="H7" s="63"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="63"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="63"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B8" s="57"/>
-      <c r="C8" s="66"/>
-      <c r="D8" s="67"/>
-      <c r="F8" s="68" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="68"/>
-      <c r="K8" s="68"/>
-      <c r="L8" s="68"/>
+      <c r="B8" s="46"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="56"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="57"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="57"/>
+      <c r="K8" s="57"/>
+      <c r="L8" s="57"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="F9" s="69"/>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="69"/>
-      <c r="J9" s="69"/>
-      <c r="K9" s="69"/>
-      <c r="L9" s="69"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="58"/>
+      <c r="J9" s="58"/>
+      <c r="K9" s="58"/>
+      <c r="L9" s="58"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="63"/>
+      <c r="F10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="64" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="65"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="K10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="50" t="s">
+      <c r="L10" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="E10" s="51"/>
-      <c r="F10" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="53"/>
-      <c r="I10" s="70"/>
-      <c r="J10" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>15</v>
       </c>
       <c r="M10" s="7"/>
     </row>
     <row r="11" spans="2:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="55"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="68"/>
       <c r="F11" s="10"/>
       <c r="G11" s="11" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="11" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J11" s="12"/>
       <c r="K11" s="13"/>
@@ -1095,35 +1025,17 @@
       <c r="M11" s="15"/>
     </row>
     <row r="12" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="16">
-        <v>27194</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="45"/>
-      <c r="F12" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="21" t="s">
-        <v>21</v>
-      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="21"/>
       <c r="H12" s="21"/>
-      <c r="I12" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J12" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="K12" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" s="22">
-        <v>12000</v>
-      </c>
+      <c r="I12" s="21"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="22"/>
       <c r="M12" s="23"/>
     </row>
     <row r="13" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
@@ -1132,34 +1044,26 @@
       <c r="D13" s="18"/>
       <c r="E13" s="19"/>
       <c r="F13" s="20"/>
-      <c r="G13" s="72" t="s">
-        <v>34</v>
-      </c>
-      <c r="H13" s="71"/>
-      <c r="I13" s="73"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="60"/>
+      <c r="I13" s="61"/>
       <c r="J13" s="20"/>
       <c r="K13" s="17"/>
-      <c r="L13" s="22">
-        <v>1000</v>
-      </c>
+      <c r="L13" s="22"/>
       <c r="M13" s="23"/>
     </row>
     <row r="14" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="16"/>
       <c r="C14" s="17"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="45"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
       <c r="F14" s="20"/>
-      <c r="G14" s="72" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="71"/>
-      <c r="I14" s="73"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="60"/>
+      <c r="I14" s="61"/>
       <c r="J14" s="20"/>
       <c r="K14" s="17"/>
-      <c r="L14" s="22">
-        <v>500</v>
-      </c>
+      <c r="L14" s="22"/>
       <c r="M14" s="23"/>
     </row>
     <row r="15" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
@@ -1168,49 +1072,33 @@
       <c r="D15" s="18"/>
       <c r="E15" s="19"/>
       <c r="F15" s="20"/>
-      <c r="G15" s="74"/>
+      <c r="G15" s="35"/>
       <c r="H15" s="35"/>
-      <c r="I15" s="74"/>
+      <c r="I15" s="35"/>
       <c r="J15" s="20"/>
       <c r="K15" s="17"/>
       <c r="L15" s="22"/>
       <c r="M15" s="23"/>
     </row>
     <row r="16" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="16">
-        <v>27195</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="45"/>
-      <c r="F16" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="21" t="s">
-        <v>21</v>
-      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="21"/>
       <c r="H16" s="21"/>
-      <c r="I16" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="20" t="s">
-        <v>23</v>
-      </c>
+      <c r="I16" s="21"/>
+      <c r="J16" s="20"/>
       <c r="K16" s="17"/>
-      <c r="L16" s="22">
-        <v>17000</v>
-      </c>
+      <c r="L16" s="22"/>
       <c r="M16" s="23"/>
     </row>
     <row r="17" spans="2:13" s="29" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B17" s="16"/>
       <c r="C17" s="17"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="45"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="44"/>
       <c r="F17" s="20"/>
       <c r="G17" s="21"/>
       <c r="H17" s="25"/>
@@ -1223,8 +1111,8 @@
     <row r="18" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="16"/>
       <c r="C18" s="17"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="45"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
       <c r="F18" s="20"/>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -1237,8 +1125,8 @@
     <row r="19" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="16"/>
       <c r="C19" s="17"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="45"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="44"/>
       <c r="F19" s="20"/>
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
@@ -1251,8 +1139,8 @@
     <row r="20" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B20" s="16"/>
       <c r="C20" s="17"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="45"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44"/>
       <c r="F20" s="20"/>
       <c r="G20" s="21"/>
       <c r="H20" s="25"/>
@@ -1265,8 +1153,8 @@
     <row r="21" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B21" s="16"/>
       <c r="C21" s="17"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
       <c r="F21" s="20"/>
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
@@ -1279,8 +1167,8 @@
     <row r="22" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B22" s="16"/>
       <c r="C22" s="17"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="44"/>
       <c r="F22" s="20"/>
       <c r="G22" s="21"/>
       <c r="H22" s="25"/>
@@ -1293,8 +1181,8 @@
     <row r="23" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="20"/>
       <c r="C23" s="31"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
       <c r="F23" s="20"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
@@ -1307,8 +1195,8 @@
     <row r="24" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B24" s="20"/>
       <c r="C24" s="31"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
       <c r="F24" s="20"/>
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
@@ -1321,8 +1209,8 @@
     <row r="25" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B25" s="20"/>
       <c r="C25" s="31"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="45"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
       <c r="F25" s="20"/>
       <c r="G25" s="21"/>
       <c r="H25" s="21"/>
@@ -1335,8 +1223,8 @@
     <row r="26" spans="2:13" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B26" s="20"/>
       <c r="C26" s="31"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="45"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="44"/>
       <c r="F26" s="33"/>
       <c r="G26" s="34"/>
       <c r="H26" s="35"/>
@@ -1347,31 +1235,24 @@
       <c r="M26" s="23"/>
     </row>
     <row r="27" spans="2:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="47"/>
-      <c r="D27" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="L27" s="37">
-        <f>SUM(L11:L26)</f>
-        <v>30500</v>
-      </c>
+      <c r="B27" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="70"/>
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="72"/>
+      <c r="K27" s="36"/>
+      <c r="L27" s="37"/>
       <c r="M27" s="38"/>
     </row>
     <row r="28" spans="2:13" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="39" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="40"/>
@@ -1394,12 +1275,12 @@
       <c r="G29" s="39"/>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
-      <c r="J29" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="K29" s="43"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
+      <c r="J29" s="73" t="s">
+        <v>15</v>
+      </c>
+      <c r="K29" s="73"/>
+      <c r="L29" s="73"/>
+      <c r="M29" s="73"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B30" s="11"/>
@@ -1431,6 +1312,19 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:J27"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:D6"/>
@@ -1446,19 +1340,6 @@
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:J27"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>